<commit_message>
feat: update task management logic and reporting formats for improved clarity and consistency
</commit_message>
<xml_diff>
--- a/phs-cr-management.report.11.17.03.07.26.output.xlsx
+++ b/phs-cr-management.report.11.17.03.07.26.output.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,12 +73,6 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00333333"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00B91C1C"/>
       <sz val="10"/>
     </font>
     <font>
@@ -140,7 +134,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -159,12 +153,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -174,7 +163,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -229,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -266,38 +255,32 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1021,7 +1004,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -1098,12 +1081,12 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -1173,12 +1156,12 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
@@ -1317,12 +1300,12 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
@@ -4317,7 +4300,7 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
@@ -4390,7 +4373,7 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -4463,7 +4446,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
@@ -6828,7 +6811,7 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -6838,29 +6821,25 @@
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>Overdue</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
           <t>UAT</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>Overdue</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>Team Mobile: overdue (deadline 31/05/2026)</t>
-        </is>
-      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="26" customHeight="1" s="5">
       <c r="A5" s="7" t="inlineStr">
@@ -6878,7 +6857,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -6888,22 +6867,22 @@
           <t>3 teams</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G5" s="16" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="I5" s="18" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>Partially Done</t>
         </is>
@@ -6917,22 +6896,22 @@
     <row r="6" ht="26" customHeight="1" s="5">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>2149046</t>
+          <t>2133352</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>EKYC</t>
+          <t>Margin product calculation tool</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>RMD</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -6940,51 +6919,47 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>Overdue</t>
-        </is>
-      </c>
-      <c r="G6" s="19" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G6" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="I6" s="12" t="inlineStr">
-        <is>
-          <t>Overdue</t>
-        </is>
-      </c>
-      <c r="J6" s="8" t="inlineStr">
-        <is>
-          <t>Team Mobile: overdue (deadline 22/05/2026)</t>
-        </is>
-      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="26" customHeight="1" s="5">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>2238356</t>
+          <t>2149046</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>ADVANCE MARGIN FOR DERIVATIVES</t>
+          <t>EKYC</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>MSD</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -6994,47 +6969,43 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Overdue</t>
-        </is>
-      </c>
-      <c r="G7" s="19" t="inlineStr">
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H7" s="13" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>Overdue</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>Team Mobile: overdue (deadline 29/05/2026)</t>
-        </is>
-      </c>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr"/>
     </row>
     <row r="8" ht="26" customHeight="1" s="5">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>2133352</t>
+          <t>2154685</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Margin product calculation tool</t>
+          <t>Upgrade fund certificate trading feature on Mobile app</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>RMD</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
+          <t>BMD</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7044,22 +7015,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G8" s="19" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
+      <c r="I8" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7069,20 +7040,20 @@
     <row r="9" ht="26" customHeight="1" s="5">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>2154685</t>
+          <t>2186435</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Upgrade fund certificate trading feature on Mobile app</t>
+          <t>PROMOTION REGISTRATION FUNCTION UPGRADE</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>BMD</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="inlineStr">
+          <t>MSD</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7092,22 +7063,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H9" s="19" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I9" s="16" t="inlineStr">
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7117,12 +7088,12 @@
     <row r="10" ht="26" customHeight="1" s="5">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>2186435</t>
+          <t>2238356</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>PROMOTION REGISTRATION FUNCTION UPGRADE</t>
+          <t>ADVANCE MARGIN FOR DERIVATIVES</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -7130,7 +7101,7 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7140,24 +7111,24 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I10" s="16" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>UAT</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr"/>
@@ -7178,7 +7149,7 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7188,22 +7159,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
       </c>
-      <c r="H11" s="19" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I11" s="17" t="inlineStr">
+      <c r="I11" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -7230,7 +7201,7 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7240,22 +7211,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H12" s="19" t="inlineStr">
+      <c r="H12" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I12" s="16" t="inlineStr">
+      <c r="I12" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7278,7 +7249,7 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7288,22 +7259,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="G13" s="19" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
+      <c r="I13" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
@@ -7330,7 +7301,7 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7340,22 +7311,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G14" s="19" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H14" s="16" t="inlineStr">
+      <c r="H14" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I14" s="16" t="inlineStr">
+      <c r="I14" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7378,7 +7349,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7388,22 +7359,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
       </c>
-      <c r="G15" s="19" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H15" s="13" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
       </c>
-      <c r="I15" s="13" t="inlineStr">
+      <c r="I15" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
@@ -7426,7 +7397,7 @@
           <t>FN</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7436,22 +7407,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F16" s="21" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G16" s="19" t="inlineStr">
+      <c r="G16" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H16" s="21" t="inlineStr">
+      <c r="H16" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="I16" s="21" t="inlineStr">
+      <c r="I16" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -7474,7 +7445,7 @@
           <t>AC</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7484,22 +7455,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="G17" s="19" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H17" s="16" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I17" s="14" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
@@ -7522,7 +7493,7 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7532,22 +7503,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F18" s="17" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="G18" s="21" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr">
+      <c r="H18" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I18" s="17" t="inlineStr">
+      <c r="I18" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -7574,7 +7545,7 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7584,22 +7555,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F19" s="21" t="inlineStr">
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="G19" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="H19" s="19" t="inlineStr">
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I19" s="17" t="inlineStr">
+      <c r="I19" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -7626,7 +7597,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7636,22 +7607,22 @@
           <t>2 teams</t>
         </is>
       </c>
-      <c r="F20" s="17" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="G20" s="21" t="inlineStr">
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="H20" s="19" t="inlineStr">
+      <c r="H20" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I20" s="17" t="inlineStr">
+      <c r="I20" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -7678,7 +7649,7 @@
           <t>BMD</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7688,22 +7659,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F21" s="19" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="G21" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H21" s="19" t="inlineStr">
+      <c r="H21" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I21" s="16" t="inlineStr">
+      <c r="I21" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7726,7 +7697,7 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7736,22 +7707,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F22" s="19" t="inlineStr">
+      <c r="F22" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G22" s="13" t="inlineStr">
+      <c r="G22" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
       </c>
-      <c r="H22" s="19" t="inlineStr">
+      <c r="H22" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr">
+      <c r="I22" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
@@ -7774,7 +7745,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7784,22 +7755,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F23" s="16" t="inlineStr">
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G23" s="19" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H23" s="19" t="inlineStr">
+      <c r="H23" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I23" s="16" t="inlineStr">
+      <c r="I23" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7822,7 +7793,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7832,22 +7803,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F24" s="16" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G24" s="19" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H24" s="19" t="inlineStr">
+      <c r="H24" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I24" s="16" t="inlineStr">
+      <c r="I24" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7870,7 +7841,7 @@
           <t>IC</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7880,22 +7851,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F25" s="16" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G25" s="19" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H25" s="19" t="inlineStr">
+      <c r="H25" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I25" s="16" t="inlineStr">
+      <c r="I25" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7918,7 +7889,7 @@
           <t>RS</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7928,22 +7899,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G26" s="19" t="inlineStr">
+      <c r="G26" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H26" s="19" t="inlineStr">
+      <c r="H26" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I26" s="16" t="inlineStr">
+      <c r="I26" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -7966,7 +7937,7 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -7976,22 +7947,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F27" s="19" t="inlineStr">
+      <c r="F27" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G27" s="14" t="inlineStr">
+      <c r="G27" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="H27" s="19" t="inlineStr">
+      <c r="H27" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I27" s="14" t="inlineStr">
+      <c r="I27" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
@@ -8014,7 +7985,7 @@
           <t>HR</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8024,22 +7995,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F28" s="19" t="inlineStr">
+      <c r="F28" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G28" s="21" t="inlineStr">
+      <c r="G28" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="H28" s="19" t="inlineStr">
+      <c r="H28" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I28" s="21" t="inlineStr">
+      <c r="I28" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -8062,7 +8033,7 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="D29" s="20" t="inlineStr">
+      <c r="D29" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8072,22 +8043,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F29" s="19" t="inlineStr">
+      <c r="F29" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G29" s="16" t="inlineStr">
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H29" s="19" t="inlineStr">
+      <c r="H29" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I29" s="16" t="inlineStr">
+      <c r="I29" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8110,7 +8081,7 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8120,22 +8091,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F30" s="16" t="inlineStr">
+      <c r="F30" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G30" s="19" t="inlineStr">
+      <c r="G30" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H30" s="19" t="inlineStr">
+      <c r="H30" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I30" s="16" t="inlineStr">
+      <c r="I30" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8158,7 +8129,7 @@
           <t>DTD</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D31" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8168,22 +8139,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F31" s="19" t="inlineStr">
+      <c r="F31" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G31" s="19" t="inlineStr">
+      <c r="G31" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H31" s="13" t="inlineStr">
+      <c r="H31" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
       </c>
-      <c r="I31" s="13" t="inlineStr">
+      <c r="I31" s="12" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
@@ -8206,7 +8177,7 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="D32" s="20" t="inlineStr">
+      <c r="D32" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8216,22 +8187,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F32" s="14" t="inlineStr">
+      <c r="F32" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="G32" s="19" t="inlineStr">
+      <c r="G32" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H32" s="19" t="inlineStr">
+      <c r="H32" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I32" s="14" t="inlineStr">
+      <c r="I32" s="13" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
@@ -8254,7 +8225,7 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="D33" s="20" t="inlineStr">
+      <c r="D33" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8264,22 +8235,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F33" s="16" t="inlineStr">
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G33" s="19" t="inlineStr">
+      <c r="G33" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H33" s="19" t="inlineStr">
+      <c r="H33" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I33" s="16" t="inlineStr">
+      <c r="I33" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8302,7 +8273,7 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="D34" s="20" t="inlineStr">
+      <c r="D34" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8312,22 +8283,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="F34" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G34" s="19" t="inlineStr">
+      <c r="G34" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H34" s="19" t="inlineStr">
+      <c r="H34" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I34" s="16" t="inlineStr">
+      <c r="I34" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8350,7 +8321,7 @@
           <t>INB</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D35" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8360,22 +8331,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="F35" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G35" s="19" t="inlineStr">
+      <c r="G35" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H35" s="19" t="inlineStr">
+      <c r="H35" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I35" s="16" t="inlineStr">
+      <c r="I35" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8398,7 +8369,7 @@
           <t>RS</t>
         </is>
       </c>
-      <c r="D36" s="20" t="inlineStr">
+      <c r="D36" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8408,22 +8379,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F36" s="19" t="inlineStr">
+      <c r="F36" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G36" s="16" t="inlineStr">
+      <c r="G36" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H36" s="19" t="inlineStr">
+      <c r="H36" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I36" s="16" t="inlineStr">
+      <c r="I36" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8446,7 +8417,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D37" s="20" t="inlineStr">
+      <c r="D37" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8456,22 +8427,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F37" s="16" t="inlineStr">
+      <c r="F37" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G37" s="19" t="inlineStr">
+      <c r="G37" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H37" s="19" t="inlineStr">
+      <c r="H37" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I37" s="16" t="inlineStr">
+      <c r="I37" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8494,7 +8465,7 @@
           <t>CCC</t>
         </is>
       </c>
-      <c r="D38" s="20" t="inlineStr">
+      <c r="D38" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8504,22 +8475,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F38" s="19" t="inlineStr">
+      <c r="F38" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G38" s="16" t="inlineStr">
+      <c r="G38" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H38" s="19" t="inlineStr">
+      <c r="H38" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I38" s="16" t="inlineStr">
+      <c r="I38" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8542,7 +8513,7 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="D39" s="20" t="inlineStr">
+      <c r="D39" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8552,22 +8523,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F39" s="16" t="inlineStr">
+      <c r="F39" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G39" s="19" t="inlineStr">
+      <c r="G39" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H39" s="19" t="inlineStr">
+      <c r="H39" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I39" s="16" t="inlineStr">
+      <c r="I39" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8590,7 +8561,7 @@
           <t>DTD</t>
         </is>
       </c>
-      <c r="D40" s="20" t="inlineStr">
+      <c r="D40" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8600,22 +8571,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F40" s="19" t="inlineStr">
+      <c r="F40" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G40" s="19" t="inlineStr">
+      <c r="G40" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H40" s="16" t="inlineStr">
+      <c r="H40" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I40" s="16" t="inlineStr">
+      <c r="I40" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8638,7 +8609,7 @@
           <t>IC</t>
         </is>
       </c>
-      <c r="D41" s="20" t="inlineStr">
+      <c r="D41" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8648,22 +8619,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F41" s="17" t="inlineStr">
+      <c r="F41" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="G41" s="19" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H41" s="19" t="inlineStr">
+      <c r="H41" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I41" s="17" t="inlineStr">
+      <c r="I41" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -8690,7 +8661,7 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="D42" s="20" t="inlineStr">
+      <c r="D42" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8700,22 +8671,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F42" s="22" t="inlineStr">
+      <c r="F42" s="20" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="G42" s="19" t="inlineStr">
+      <c r="G42" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H42" s="19" t="inlineStr">
+      <c r="H42" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I42" s="22" t="inlineStr">
+      <c r="I42" s="20" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -8734,7 +8705,7 @@
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr"/>
-      <c r="D43" s="20" t="inlineStr">
+      <c r="D43" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8744,22 +8715,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F43" s="16" t="inlineStr">
+      <c r="F43" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G43" s="19" t="inlineStr">
+      <c r="G43" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H43" s="19" t="inlineStr">
+      <c r="H43" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I43" s="16" t="inlineStr">
+      <c r="I43" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8782,7 +8753,7 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="D44" s="20" t="inlineStr">
+      <c r="D44" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8792,22 +8763,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F44" s="21" t="inlineStr">
+      <c r="F44" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G44" s="19" t="inlineStr">
+      <c r="G44" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H44" s="19" t="inlineStr">
+      <c r="H44" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I44" s="21" t="inlineStr">
+      <c r="I44" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -8830,7 +8801,7 @@
           <t>AC</t>
         </is>
       </c>
-      <c r="D45" s="20" t="inlineStr">
+      <c r="D45" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8840,22 +8811,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F45" s="17" t="inlineStr">
+      <c r="F45" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="G45" s="19" t="inlineStr">
+      <c r="G45" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H45" s="19" t="inlineStr">
+      <c r="H45" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I45" s="17" t="inlineStr">
+      <c r="I45" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -8882,7 +8853,7 @@
           <t>FN</t>
         </is>
       </c>
-      <c r="D46" s="20" t="inlineStr">
+      <c r="D46" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8892,22 +8863,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F46" s="19" t="inlineStr">
+      <c r="F46" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G46" s="19" t="inlineStr">
+      <c r="G46" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H46" s="16" t="inlineStr">
+      <c r="H46" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I46" s="16" t="inlineStr">
+      <c r="I46" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8926,7 +8897,7 @@
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr"/>
-      <c r="D47" s="20" t="inlineStr">
+      <c r="D47" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8936,22 +8907,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F47" s="16" t="inlineStr">
+      <c r="F47" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G47" s="19" t="inlineStr">
+      <c r="G47" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H47" s="19" t="inlineStr">
+      <c r="H47" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I47" s="16" t="inlineStr">
+      <c r="I47" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -8974,7 +8945,7 @@
           <t>CCC</t>
         </is>
       </c>
-      <c r="D48" s="20" t="inlineStr">
+      <c r="D48" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8984,22 +8955,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F48" s="21" t="inlineStr">
+      <c r="F48" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G48" s="19" t="inlineStr">
+      <c r="G48" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H48" s="19" t="inlineStr">
+      <c r="H48" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I48" s="21" t="inlineStr">
+      <c r="I48" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -9022,7 +8993,7 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="D49" s="20" t="inlineStr">
+      <c r="D49" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9032,22 +9003,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F49" s="19" t="inlineStr">
+      <c r="F49" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G49" s="16" t="inlineStr">
+      <c r="G49" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H49" s="19" t="inlineStr">
+      <c r="H49" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I49" s="16" t="inlineStr">
+      <c r="I49" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9070,7 +9041,7 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="D50" s="20" t="inlineStr">
+      <c r="D50" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9080,22 +9051,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F50" s="21" t="inlineStr">
+      <c r="F50" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G50" s="19" t="inlineStr">
+      <c r="G50" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H50" s="19" t="inlineStr">
+      <c r="H50" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I50" s="21" t="inlineStr">
+      <c r="I50" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -9114,7 +9085,7 @@
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr"/>
-      <c r="D51" s="20" t="inlineStr">
+      <c r="D51" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9124,22 +9095,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F51" s="16" t="inlineStr">
+      <c r="F51" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G51" s="19" t="inlineStr">
+      <c r="G51" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H51" s="19" t="inlineStr">
+      <c r="H51" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I51" s="16" t="inlineStr">
+      <c r="I51" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9162,7 +9133,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D52" s="20" t="inlineStr">
+      <c r="D52" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9172,22 +9143,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F52" s="19" t="inlineStr">
+      <c r="F52" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G52" s="17" t="inlineStr">
+      <c r="G52" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="H52" s="19" t="inlineStr">
+      <c r="H52" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I52" s="17" t="inlineStr">
+      <c r="I52" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -9214,7 +9185,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D53" s="20" t="inlineStr">
+      <c r="D53" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9224,22 +9195,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F53" s="19" t="inlineStr">
+      <c r="F53" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G53" s="16" t="inlineStr">
+      <c r="G53" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="H53" s="19" t="inlineStr">
+      <c r="H53" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I53" s="16" t="inlineStr">
+      <c r="I53" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9262,7 +9233,7 @@
           <t>RS</t>
         </is>
       </c>
-      <c r="D54" s="20" t="inlineStr">
+      <c r="D54" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9272,22 +9243,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F54" s="19" t="inlineStr">
+      <c r="F54" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G54" s="21" t="inlineStr">
+      <c r="G54" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="H54" s="19" t="inlineStr">
+      <c r="H54" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I54" s="21" t="inlineStr">
+      <c r="I54" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -9310,7 +9281,7 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="D55" s="20" t="inlineStr">
+      <c r="D55" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9320,22 +9291,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F55" s="19" t="inlineStr">
+      <c r="F55" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G55" s="17" t="inlineStr">
+      <c r="G55" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="H55" s="19" t="inlineStr">
+      <c r="H55" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I55" s="17" t="inlineStr">
+      <c r="I55" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -9362,7 +9333,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D56" s="20" t="inlineStr">
+      <c r="D56" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9372,22 +9343,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F56" s="19" t="inlineStr">
+      <c r="F56" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G56" s="19" t="inlineStr">
+      <c r="G56" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H56" s="17" t="inlineStr">
+      <c r="H56" s="15" t="inlineStr">
         <is>
           <t>Doing</t>
         </is>
       </c>
-      <c r="I56" s="17" t="inlineStr">
+      <c r="I56" s="15" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -9414,7 +9385,7 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="D57" s="20" t="inlineStr">
+      <c r="D57" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9424,22 +9395,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F57" s="21" t="inlineStr">
+      <c r="F57" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G57" s="19" t="inlineStr">
+      <c r="G57" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H57" s="19" t="inlineStr">
+      <c r="H57" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I57" s="21" t="inlineStr">
+      <c r="I57" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -9462,7 +9433,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D58" s="20" t="inlineStr">
+      <c r="D58" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9472,22 +9443,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F58" s="19" t="inlineStr">
+      <c r="F58" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G58" s="19" t="inlineStr">
+      <c r="G58" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H58" s="16" t="inlineStr">
+      <c r="H58" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I58" s="16" t="inlineStr">
+      <c r="I58" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9510,7 +9481,7 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="D59" s="20" t="inlineStr">
+      <c r="D59" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9520,22 +9491,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F59" s="19" t="inlineStr">
+      <c r="F59" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G59" s="19" t="inlineStr">
+      <c r="G59" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H59" s="16" t="inlineStr">
+      <c r="H59" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I59" s="16" t="inlineStr">
+      <c r="I59" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9558,7 +9529,7 @@
           <t>AC</t>
         </is>
       </c>
-      <c r="D60" s="20" t="inlineStr">
+      <c r="D60" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9568,22 +9539,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F60" s="21" t="inlineStr">
+      <c r="F60" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G60" s="19" t="inlineStr">
+      <c r="G60" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H60" s="19" t="inlineStr">
+      <c r="H60" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I60" s="21" t="inlineStr">
+      <c r="I60" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -9606,7 +9577,7 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="D61" s="20" t="inlineStr">
+      <c r="D61" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9616,22 +9587,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F61" s="21" t="inlineStr">
+      <c r="F61" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G61" s="19" t="inlineStr">
+      <c r="G61" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H61" s="19" t="inlineStr">
+      <c r="H61" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I61" s="21" t="inlineStr">
+      <c r="I61" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -9654,7 +9625,7 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="D62" s="20" t="inlineStr">
+      <c r="D62" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9664,22 +9635,22 @@
           <t>1 team</t>
         </is>
       </c>
-      <c r="F62" s="21" t="inlineStr">
+      <c r="F62" s="19" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="G62" s="19" t="inlineStr">
+      <c r="G62" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H62" s="19" t="inlineStr">
+      <c r="H62" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I62" s="21" t="inlineStr">
+      <c r="I62" s="19" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
@@ -9687,107 +9658,107 @@
       <c r="J62" s="8" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="23" t="inlineStr">
+      <c r="A64" s="21" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="24" t="inlineStr">
+      <c r="A65" s="22" t="inlineStr">
         <is>
           <t>Total unique CRs:</t>
         </is>
       </c>
-      <c r="B65" s="25">
+      <c r="B65" s="23">
         <f>COUNTA(A4:A62)</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="24" t="inlineStr">
+      <c r="A66" s="22" t="inlineStr">
         <is>
           <t>Multi-team CRs:</t>
         </is>
       </c>
-      <c r="B66" s="25">
+      <c r="B66" s="23">
         <f>COUNTIF(E4:E62,"2 teams")+COUNTIF(E4:E62,"3 teams")</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="24" t="inlineStr">
+      <c r="A67" s="22" t="inlineStr">
         <is>
           <t>CRs with Overdue status:</t>
         </is>
       </c>
-      <c r="B67" s="25">
+      <c r="B67" s="23">
         <f>COUNTIF(I4:I62,"Overdue")</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="24" t="inlineStr">
+      <c r="A68" s="22" t="inlineStr">
         <is>
           <t>CRs fully Done:</t>
         </is>
       </c>
-      <c r="B68" s="25">
+      <c r="B68" s="23">
         <f>COUNTIF(I4:I62,"Done")</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="24" t="inlineStr">
+      <c r="A69" s="22" t="inlineStr">
         <is>
           <t>CRs Partially Done:</t>
         </is>
       </c>
-      <c r="B69" s="25">
+      <c r="B69" s="23">
         <f>COUNTIF(I4:I62,"Partially Done")</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="24" t="inlineStr">
+      <c r="A70" s="22" t="inlineStr">
         <is>
           <t>CRs In Progress:</t>
         </is>
       </c>
-      <c r="B70" s="25">
+      <c r="B70" s="23">
         <f>COUNTIF(I4:I62,"In Progress")</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="24" t="inlineStr">
+      <c r="A71" s="22" t="inlineStr">
         <is>
           <t>CRs in UAT:</t>
         </is>
       </c>
-      <c r="B71" s="25">
+      <c r="B71" s="23">
         <f>COUNTIF(I4:I62,"UAT")</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="24" t="inlineStr">
+      <c r="A72" s="22" t="inlineStr">
         <is>
           <t>CRs Blocked:</t>
         </is>
       </c>
-      <c r="B72" s="25">
+      <c r="B72" s="23">
         <f>COUNTIF(I4:I62,"Blocked")</f>
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="24" t="inlineStr">
+      <c r="A73" s="22" t="inlineStr">
         <is>
           <t>CRs Rejected:</t>
         </is>
       </c>
-      <c r="B73" s="25">
+      <c r="B73" s="23">
         <f>COUNTIF(I4:I62,"Rejected")</f>
         <v/>
       </c>
@@ -9811,147 +9782,147 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>report_date</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>task_id</t>
         </is>
       </c>
-      <c r="C1" s="26" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>request_id</t>
         </is>
       </c>
-      <c r="D1" s="26" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="E1" s="26" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>assignee</t>
         </is>
       </c>
-      <c r="F1" s="26" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="G1" s="26" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>stage_order</t>
         </is>
       </c>
-      <c r="H1" s="26" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="I1" s="26" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="J1" s="26" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>phase</t>
         </is>
       </c>
-      <c r="K1" s="26" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>q_kpi</t>
         </is>
       </c>
-      <c r="L1" s="26" t="inlineStr">
+      <c r="L1" s="24" t="inlineStr">
         <is>
           <t>is_subtask</t>
         </is>
       </c>
-      <c r="M1" s="26" t="inlineStr">
+      <c r="M1" s="24" t="inlineStr">
         <is>
           <t>is_done</t>
         </is>
       </c>
-      <c r="N1" s="26" t="inlineStr">
+      <c r="N1" s="24" t="inlineStr">
         <is>
           <t>wip_flag</t>
         </is>
       </c>
-      <c r="O1" s="26" t="inlineStr">
+      <c r="O1" s="24" t="inlineStr">
         <is>
           <t>is_multi_team</t>
         </is>
       </c>
-      <c r="P1" s="26" t="inlineStr">
+      <c r="P1" s="24" t="inlineStr">
         <is>
           <t>team_count</t>
         </is>
       </c>
-      <c r="Q1" s="26" t="inlineStr">
+      <c r="Q1" s="24" t="inlineStr">
         <is>
           <t>has_deadline</t>
         </is>
       </c>
-      <c r="R1" s="26" t="inlineStr">
+      <c r="R1" s="24" t="inlineStr">
         <is>
           <t>sla_met</t>
         </is>
       </c>
-      <c r="S1" s="26" t="inlineStr">
+      <c r="S1" s="24" t="inlineStr">
         <is>
           <t>completed_late</t>
         </is>
       </c>
-      <c r="T1" s="26" t="inlineStr">
+      <c r="T1" s="24" t="inlineStr">
         <is>
           <t>late_days</t>
         </is>
       </c>
-      <c r="U1" s="26" t="inlineStr">
+      <c r="U1" s="24" t="inlineStr">
         <is>
           <t>days_to_deadline</t>
         </is>
       </c>
-      <c r="V1" s="26" t="inlineStr">
+      <c r="V1" s="24" t="inlineStr">
         <is>
           <t>age_days</t>
         </is>
       </c>
-      <c r="W1" s="26" t="inlineStr">
+      <c r="W1" s="24" t="inlineStr">
         <is>
           <t>cycle_time_days</t>
         </is>
       </c>
-      <c r="X1" s="26" t="inlineStr">
+      <c r="X1" s="24" t="inlineStr">
         <is>
           <t>lead_time_days</t>
         </is>
       </c>
-      <c r="Y1" s="26" t="inlineStr">
+      <c r="Y1" s="24" t="inlineStr">
         <is>
           <t>stale_days</t>
         </is>
       </c>
-      <c r="Z1" s="26" t="inlineStr">
+      <c r="Z1" s="24" t="inlineStr">
         <is>
           <t>risk_level</t>
         </is>
       </c>
-      <c r="AA1" s="26" t="inlineStr">
+      <c r="AA1" s="24" t="inlineStr">
         <is>
           <t>waiting_external</t>
         </is>
       </c>
-      <c r="AB1" s="26" t="inlineStr">
+      <c r="AB1" s="24" t="inlineStr">
         <is>
           <t>has_weekly_review</t>
         </is>
       </c>
-      <c r="AC1" s="26" t="inlineStr">
+      <c r="AC1" s="24" t="inlineStr">
         <is>
           <t>recommit_count</t>
         </is>
@@ -10289,7 +10260,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -10389,12 +10360,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -10414,7 +10385,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" t="b">
         <v>1</v>
@@ -10491,12 +10462,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -10516,7 +10487,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" t="b">
         <v>1</v>
@@ -10688,12 +10659,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -10713,7 +10684,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" t="b">
         <v>1</v>
@@ -14757,7 +14728,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -14852,7 +14823,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -14947,7 +14918,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -18124,97 +18095,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>task_id</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>request_id</t>
         </is>
       </c>
-      <c r="C1" s="26" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>task_name</t>
         </is>
       </c>
-      <c r="D1" s="26" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" s="26" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>dept_tag</t>
         </is>
       </c>
-      <c r="F1" s="26" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>metatype</t>
         </is>
       </c>
-      <c r="G1" s="26" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>parent_id</t>
         </is>
       </c>
-      <c r="H1" s="26" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>jira_url</t>
         </is>
       </c>
-      <c r="I1" s="26" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>owner_division</t>
         </is>
       </c>
-      <c r="J1" s="26" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="K1" s="26" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>start_at</t>
         </is>
       </c>
-      <c r="L1" s="26" t="inlineStr">
+      <c r="L1" s="24" t="inlineStr">
         <is>
           <t>deadline_at</t>
         </is>
       </c>
-      <c r="M1" s="26" t="inlineStr">
+      <c r="M1" s="24" t="inlineStr">
         <is>
           <t>completed_at</t>
         </is>
       </c>
-      <c r="N1" s="26" t="inlineStr">
+      <c r="N1" s="24" t="inlineStr">
         <is>
           <t>cr_received</t>
         </is>
       </c>
-      <c r="O1" s="26" t="inlineStr">
+      <c r="O1" s="24" t="inlineStr">
         <is>
           <t>cr_recommit</t>
         </is>
       </c>
-      <c r="P1" s="26" t="inlineStr">
+      <c r="P1" s="24" t="inlineStr">
         <is>
           <t>last_review</t>
         </is>
       </c>
-      <c r="Q1" s="26" t="inlineStr">
+      <c r="Q1" s="24" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="R1" s="26" t="inlineStr">
+      <c r="R1" s="24" t="inlineStr">
         <is>
           <t>wr_assessment</t>
         </is>
       </c>
-      <c r="S1" s="26" t="inlineStr">
+      <c r="S1" s="24" t="inlineStr">
         <is>
           <t>wr_next</t>
         </is>
@@ -18250,7 +18221,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="27" t="n">
+      <c r="J2" s="25" t="n">
         <v>46206.43125</v>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -18303,19 +18274,19 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J3" s="27" t="n">
+      <c r="J3" s="25" t="n">
         <v>46192.40208333333</v>
       </c>
-      <c r="L3" s="27" t="n">
+      <c r="L3" s="25" t="n">
         <v>46202.99930555555</v>
       </c>
-      <c r="M3" s="27" t="n">
+      <c r="M3" s="25" t="n">
         <v>46205.66875</v>
       </c>
-      <c r="N3" s="27" t="n">
+      <c r="N3" s="25" t="n">
         <v>45946</v>
       </c>
-      <c r="O3" s="27" t="n">
+      <c r="O3" s="25" t="n">
         <v>46149</v>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -18368,19 +18339,19 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J4" s="27" t="n">
+      <c r="J4" s="25" t="n">
         <v>46181.57638888889</v>
       </c>
-      <c r="L4" s="27" t="n">
+      <c r="L4" s="25" t="n">
         <v>46185.99930555555</v>
       </c>
-      <c r="M4" s="27" t="n">
+      <c r="M4" s="25" t="n">
         <v>46185.34444444445</v>
       </c>
-      <c r="N4" s="27" t="n">
+      <c r="N4" s="25" t="n">
         <v>46118</v>
       </c>
-      <c r="O4" s="27" t="n">
+      <c r="O4" s="25" t="n">
         <v>46167</v>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -18433,19 +18404,19 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J5" s="27" t="n">
+      <c r="J5" s="25" t="n">
         <v>46147.73402777778</v>
       </c>
-      <c r="L5" s="27" t="n">
+      <c r="L5" s="25" t="n">
         <v>46157.99930555555</v>
       </c>
-      <c r="M5" s="27" t="n">
+      <c r="M5" s="25" t="n">
         <v>46158.33402777778</v>
       </c>
-      <c r="N5" s="27" t="n">
+      <c r="N5" s="25" t="n">
         <v>45934</v>
       </c>
-      <c r="O5" s="27" t="n">
+      <c r="O5" s="25" t="n">
         <v>46049</v>
       </c>
       <c r="Q5" t="inlineStr"/>
@@ -18498,22 +18469,22 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J6" s="27" t="n">
+      <c r="J6" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="K6" s="27" t="n">
+      <c r="K6" s="25" t="n">
         <v>46055</v>
       </c>
-      <c r="L6" s="27" t="n">
+      <c r="L6" s="25" t="n">
         <v>46173.99930555555</v>
       </c>
-      <c r="N6" s="27" t="n">
+      <c r="N6" s="25" t="n">
         <v>45934</v>
       </c>
-      <c r="O6" s="27" t="n">
+      <c r="O6" s="25" t="n">
         <v>46064</v>
       </c>
-      <c r="P6" s="27" t="n">
+      <c r="P6" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -18574,13 +18545,13 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="J7" s="27" t="n">
+      <c r="J7" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="L7" s="27" t="n">
+      <c r="L7" s="25" t="n">
         <v>46164.99930555555</v>
       </c>
-      <c r="P7" s="27" t="n">
+      <c r="P7" s="25" t="n">
         <v>46203</v>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -18641,13 +18612,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J8" s="27" t="n">
+      <c r="J8" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="N8" s="27" t="n">
+      <c r="N8" s="25" t="n">
         <v>46049</v>
       </c>
-      <c r="P8" s="27" t="n">
+      <c r="P8" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -18708,19 +18679,19 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J9" s="27" t="n">
+      <c r="J9" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="K9" s="27" t="n">
+      <c r="K9" s="25" t="n">
         <v>46093</v>
       </c>
-      <c r="L9" s="27" t="n">
+      <c r="L9" s="25" t="n">
         <v>46171.99930555555</v>
       </c>
-      <c r="N9" s="27" t="n">
+      <c r="N9" s="25" t="n">
         <v>46017</v>
       </c>
-      <c r="P9" s="27" t="n">
+      <c r="P9" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q9" t="inlineStr"/>
@@ -18777,13 +18748,13 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J10" s="27" t="n">
+      <c r="J10" s="25" t="n">
         <v>46125.72361111111</v>
       </c>
-      <c r="N10" s="27" t="n">
+      <c r="N10" s="25" t="n">
         <v>46118</v>
       </c>
-      <c r="P10" s="27" t="n">
+      <c r="P10" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -18840,10 +18811,10 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J11" s="27" t="n">
+      <c r="J11" s="25" t="n">
         <v>46205.37222222222</v>
       </c>
-      <c r="N11" s="27" t="n">
+      <c r="N11" s="25" t="n">
         <v>46104</v>
       </c>
       <c r="Q11" t="inlineStr"/>
@@ -18892,10 +18863,10 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="J12" s="27" t="n">
+      <c r="J12" s="25" t="n">
         <v>46205.37152777778</v>
       </c>
-      <c r="N12" s="27" t="n">
+      <c r="N12" s="25" t="n">
         <v>46128</v>
       </c>
       <c r="Q12" t="inlineStr"/>
@@ -18944,10 +18915,10 @@
           <t>RS</t>
         </is>
       </c>
-      <c r="J13" s="27" t="n">
+      <c r="J13" s="25" t="n">
         <v>46205.37152777778</v>
       </c>
-      <c r="N13" s="27" t="n">
+      <c r="N13" s="25" t="n">
         <v>46135</v>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -18996,10 +18967,10 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="J14" s="27" t="n">
+      <c r="J14" s="25" t="n">
         <v>46205.36388888889</v>
       </c>
-      <c r="N14" s="27" t="n">
+      <c r="N14" s="25" t="n">
         <v>46136</v>
       </c>
       <c r="Q14" t="inlineStr"/>
@@ -19048,13 +19019,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J15" s="27" t="n">
+      <c r="J15" s="25" t="n">
         <v>46205.3625</v>
       </c>
-      <c r="N15" s="27" t="n">
+      <c r="N15" s="25" t="n">
         <v>46022</v>
       </c>
-      <c r="O15" s="27" t="n">
+      <c r="O15" s="25" t="n">
         <v>46156</v>
       </c>
       <c r="Q15" t="inlineStr"/>
@@ -19103,7 +19074,7 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J16" s="27" t="n">
+      <c r="J16" s="25" t="n">
         <v>46205.3625</v>
       </c>
       <c r="Q16" t="inlineStr"/>
@@ -19152,7 +19123,7 @@
           <t>HR</t>
         </is>
       </c>
-      <c r="J17" s="27" t="n">
+      <c r="J17" s="25" t="n">
         <v>46148.35694444444</v>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -19205,7 +19176,7 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J18" s="27" t="n">
+      <c r="J18" s="25" t="n">
         <v>46126.39236111111</v>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -19254,16 +19225,16 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J19" s="27" t="n">
+      <c r="J19" s="25" t="n">
         <v>46148.57916666667</v>
       </c>
-      <c r="N19" s="27" t="n">
+      <c r="N19" s="25" t="n">
         <v>46022</v>
       </c>
-      <c r="O19" s="27" t="n">
+      <c r="O19" s="25" t="n">
         <v>46156</v>
       </c>
-      <c r="P19" s="27" t="n">
+      <c r="P19" s="25" t="n">
         <v>46205</v>
       </c>
       <c r="Q19" t="inlineStr"/>
@@ -19324,19 +19295,19 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J20" s="27" t="n">
+      <c r="J20" s="25" t="n">
         <v>46126.38680555556</v>
       </c>
-      <c r="L20" s="27" t="n">
+      <c r="L20" s="25" t="n">
         <v>46146.99930555555</v>
       </c>
-      <c r="M20" s="27" t="n">
+      <c r="M20" s="25" t="n">
         <v>46147.73819444444</v>
       </c>
-      <c r="N20" s="27" t="n">
+      <c r="N20" s="25" t="n">
         <v>46049</v>
       </c>
-      <c r="O20" s="27" t="n">
+      <c r="O20" s="25" t="n">
         <v>46136</v>
       </c>
       <c r="Q20" t="inlineStr"/>
@@ -19389,16 +19360,16 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="J21" s="27" t="n">
+      <c r="J21" s="25" t="n">
         <v>46126.40486111111</v>
       </c>
-      <c r="L21" s="27" t="n">
+      <c r="L21" s="25" t="n">
         <v>46199.99930555555</v>
       </c>
-      <c r="M21" s="27" t="n">
+      <c r="M21" s="25" t="n">
         <v>46202.34513888889</v>
       </c>
-      <c r="N21" s="27" t="n">
+      <c r="N21" s="25" t="n">
         <v>46125</v>
       </c>
       <c r="Q21" t="inlineStr"/>
@@ -19451,13 +19422,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J22" s="27" t="n">
+      <c r="J22" s="25" t="n">
         <v>46147.74166666667</v>
       </c>
-      <c r="M22" s="27" t="n">
+      <c r="M22" s="25" t="n">
         <v>46174.34097222222</v>
       </c>
-      <c r="N22" s="27" t="n">
+      <c r="N22" s="25" t="n">
         <v>46146</v>
       </c>
       <c r="Q22" t="inlineStr"/>
@@ -19510,22 +19481,22 @@
           <t>BMD</t>
         </is>
       </c>
-      <c r="J23" s="27" t="n">
+      <c r="J23" s="25" t="n">
         <v>46126.38541666666</v>
       </c>
-      <c r="K23" s="27" t="n">
+      <c r="K23" s="25" t="n">
         <v>46062</v>
       </c>
-      <c r="L23" s="27" t="n">
+      <c r="L23" s="25" t="n">
         <v>46140.99930555555</v>
       </c>
-      <c r="M23" s="27" t="n">
+      <c r="M23" s="25" t="n">
         <v>46147.60833333333</v>
       </c>
-      <c r="N23" s="27" t="n">
+      <c r="N23" s="25" t="n">
         <v>45972</v>
       </c>
-      <c r="O23" s="27" t="n">
+      <c r="O23" s="25" t="n">
         <v>46049</v>
       </c>
       <c r="Q23" t="inlineStr"/>
@@ -19578,16 +19549,16 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="J24" s="27" t="n">
+      <c r="J24" s="25" t="n">
         <v>46126.38541666666</v>
       </c>
-      <c r="M24" s="27" t="n">
+      <c r="M24" s="25" t="n">
         <v>46137.38680555556</v>
       </c>
-      <c r="N24" s="27" t="n">
+      <c r="N24" s="25" t="n">
         <v>46108</v>
       </c>
-      <c r="O24" s="27" t="n">
+      <c r="O24" s="25" t="n">
         <v>46118</v>
       </c>
       <c r="Q24" t="inlineStr"/>
@@ -19640,19 +19611,19 @@
           <t>RS</t>
         </is>
       </c>
-      <c r="J25" s="27" t="n">
+      <c r="J25" s="25" t="n">
         <v>46126.38611111111</v>
       </c>
-      <c r="K25" s="27" t="n">
+      <c r="K25" s="25" t="n">
         <v>46090</v>
       </c>
-      <c r="M25" s="27" t="n">
+      <c r="M25" s="25" t="n">
         <v>46132.35277777778</v>
       </c>
-      <c r="N25" s="27" t="n">
+      <c r="N25" s="25" t="n">
         <v>45993</v>
       </c>
-      <c r="O25" s="27" t="n">
+      <c r="O25" s="25" t="n">
         <v>46076</v>
       </c>
       <c r="Q25" t="inlineStr"/>
@@ -19705,10 +19676,10 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="J26" s="27" t="n">
+      <c r="J26" s="25" t="n">
         <v>46204.39930555555</v>
       </c>
-      <c r="N26" s="27" t="n">
+      <c r="N26" s="25" t="n">
         <v>46203</v>
       </c>
       <c r="Q26" t="inlineStr"/>
@@ -19761,10 +19732,10 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="J27" s="27" t="n">
+      <c r="J27" s="25" t="n">
         <v>46204.39930555555</v>
       </c>
-      <c r="N27" s="27" t="n">
+      <c r="N27" s="25" t="n">
         <v>46203</v>
       </c>
       <c r="Q27" t="inlineStr"/>
@@ -19817,13 +19788,13 @@
           <t>ACC</t>
         </is>
       </c>
-      <c r="J28" s="27" t="n">
+      <c r="J28" s="25" t="n">
         <v>46178.40902777778</v>
       </c>
-      <c r="N28" s="27" t="n">
+      <c r="N28" s="25" t="n">
         <v>46174</v>
       </c>
-      <c r="P28" s="27" t="n">
+      <c r="P28" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q28" t="inlineStr"/>
@@ -19884,10 +19855,10 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J29" s="27" t="n">
+      <c r="J29" s="25" t="n">
         <v>46204.39861111111</v>
       </c>
-      <c r="N29" s="27" t="n">
+      <c r="N29" s="25" t="n">
         <v>46022</v>
       </c>
       <c r="Q29" t="inlineStr"/>
@@ -19940,10 +19911,10 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J30" s="27" t="n">
+      <c r="J30" s="25" t="n">
         <v>46204.39791666667</v>
       </c>
-      <c r="N30" s="27" t="n">
+      <c r="N30" s="25" t="n">
         <v>46203</v>
       </c>
       <c r="Q30" t="inlineStr"/>
@@ -19996,13 +19967,13 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="J31" s="27" t="n">
+      <c r="J31" s="25" t="n">
         <v>46178.40763888889</v>
       </c>
-      <c r="N31" s="27" t="n">
+      <c r="N31" s="25" t="n">
         <v>46128</v>
       </c>
-      <c r="P31" s="27" t="n">
+      <c r="P31" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q31" t="inlineStr"/>
@@ -20063,10 +20034,10 @@
           <t>ACC</t>
         </is>
       </c>
-      <c r="J32" s="27" t="n">
+      <c r="J32" s="25" t="n">
         <v>46204.39791666667</v>
       </c>
-      <c r="N32" s="27" t="n">
+      <c r="N32" s="25" t="n">
         <v>46107</v>
       </c>
       <c r="Q32" t="inlineStr"/>
@@ -20119,13 +20090,13 @@
           <t>IC</t>
         </is>
       </c>
-      <c r="J33" s="27" t="n">
+      <c r="J33" s="25" t="n">
         <v>46178.4125</v>
       </c>
-      <c r="N33" s="27" t="n">
+      <c r="N33" s="25" t="n">
         <v>46129</v>
       </c>
-      <c r="P33" s="27" t="n">
+      <c r="P33" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -20186,13 +20157,13 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="J34" s="27" t="n">
+      <c r="J34" s="25" t="n">
         <v>46125.72291666667</v>
       </c>
-      <c r="N34" s="27" t="n">
+      <c r="N34" s="25" t="n">
         <v>46118</v>
       </c>
-      <c r="P34" s="27" t="n">
+      <c r="P34" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q34" t="inlineStr"/>
@@ -20253,13 +20224,13 @@
           <t>AC</t>
         </is>
       </c>
-      <c r="J35" s="27" t="n">
+      <c r="J35" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="N35" s="27" t="n">
+      <c r="N35" s="25" t="n">
         <v>46077</v>
       </c>
-      <c r="P35" s="27" t="n">
+      <c r="P35" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q35" t="inlineStr"/>
@@ -20320,13 +20291,13 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J36" s="27" t="n">
+      <c r="J36" s="25" t="n">
         <v>46125.71597222222</v>
       </c>
-      <c r="N36" s="27" t="n">
+      <c r="N36" s="25" t="n">
         <v>46104</v>
       </c>
-      <c r="P36" s="27" t="n">
+      <c r="P36" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q36" t="inlineStr"/>
@@ -20387,10 +20358,10 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="J37" s="27" t="n">
+      <c r="J37" s="25" t="n">
         <v>46204.39861111111</v>
       </c>
-      <c r="N37" s="27" t="n">
+      <c r="N37" s="25" t="n">
         <v>46153</v>
       </c>
       <c r="Q37" t="inlineStr"/>
@@ -20443,13 +20414,13 @@
           <t>FN</t>
         </is>
       </c>
-      <c r="J38" s="27" t="n">
+      <c r="J38" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="N38" s="27" t="n">
+      <c r="N38" s="25" t="n">
         <v>46052</v>
       </c>
-      <c r="P38" s="27" t="n">
+      <c r="P38" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q38" t="inlineStr"/>
@@ -20510,13 +20481,13 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="J39" s="27" t="n">
+      <c r="J39" s="25" t="n">
         <v>46125.72083333333</v>
       </c>
-      <c r="N39" s="27" t="n">
+      <c r="N39" s="25" t="n">
         <v>46097</v>
       </c>
-      <c r="P39" s="27" t="n">
+      <c r="P39" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q39" t="inlineStr"/>
@@ -20577,13 +20548,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J40" s="27" t="n">
+      <c r="J40" s="25" t="n">
         <v>46125.72222222222</v>
       </c>
-      <c r="N40" s="27" t="n">
+      <c r="N40" s="25" t="n">
         <v>46108</v>
       </c>
-      <c r="P40" s="27" t="n">
+      <c r="P40" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q40" t="inlineStr"/>
@@ -20644,13 +20615,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J41" s="27" t="n">
+      <c r="J41" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="N41" s="27" t="n">
+      <c r="N41" s="25" t="n">
         <v>46047</v>
       </c>
-      <c r="P41" s="27" t="n">
+      <c r="P41" s="25" t="n">
         <v>46204</v>
       </c>
       <c r="Q41" t="inlineStr"/>
@@ -20707,13 +20678,13 @@
           <t>FN</t>
         </is>
       </c>
-      <c r="J42" s="27" t="n">
+      <c r="J42" s="25" t="n">
         <v>46179.6625</v>
       </c>
-      <c r="M42" s="27" t="n">
+      <c r="M42" s="25" t="n">
         <v>46179.66388888889</v>
       </c>
-      <c r="N42" s="27" t="n">
+      <c r="N42" s="25" t="n">
         <v>46083</v>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -20762,13 +20733,13 @@
           <t>ACC</t>
         </is>
       </c>
-      <c r="J43" s="27" t="n">
+      <c r="J43" s="25" t="n">
         <v>46154.37708333333</v>
       </c>
-      <c r="M43" s="27" t="n">
+      <c r="M43" s="25" t="n">
         <v>46205.70138888889</v>
       </c>
-      <c r="N43" s="27" t="n">
+      <c r="N43" s="25" t="n">
         <v>46107</v>
       </c>
       <c r="Q43" t="inlineStr"/>
@@ -20821,16 +20792,16 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J44" s="27" t="n">
+      <c r="J44" s="25" t="n">
         <v>46154.38125</v>
       </c>
-      <c r="M44" s="27" t="n">
+      <c r="M44" s="25" t="n">
         <v>46189.43402777778</v>
       </c>
-      <c r="N44" s="27" t="n">
+      <c r="N44" s="25" t="n">
         <v>46149</v>
       </c>
-      <c r="O44" s="27" t="n">
+      <c r="O44" s="25" t="n">
         <v>46164</v>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -20883,13 +20854,13 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J45" s="27" t="n">
+      <c r="J45" s="25" t="n">
         <v>46154.375</v>
       </c>
-      <c r="M45" s="27" t="n">
+      <c r="M45" s="25" t="n">
         <v>46155.43541666667</v>
       </c>
-      <c r="N45" s="27" t="n">
+      <c r="N45" s="25" t="n">
         <v>46003</v>
       </c>
       <c r="Q45" t="inlineStr"/>
@@ -20938,13 +20909,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J46" s="27" t="n">
+      <c r="J46" s="25" t="n">
         <v>46154.38472222222</v>
       </c>
-      <c r="M46" s="27" t="n">
+      <c r="M46" s="25" t="n">
         <v>46178.4625</v>
       </c>
-      <c r="N46" s="27" t="n">
+      <c r="N46" s="25" t="n">
         <v>46148</v>
       </c>
       <c r="Q46" t="inlineStr"/>
@@ -20997,13 +20968,13 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J47" s="27" t="n">
+      <c r="J47" s="25" t="n">
         <v>46154.36319444444</v>
       </c>
-      <c r="M47" s="27" t="n">
+      <c r="M47" s="25" t="n">
         <v>46157.43888888889</v>
       </c>
-      <c r="N47" s="27" t="n">
+      <c r="N47" s="25" t="n">
         <v>45952</v>
       </c>
       <c r="Q47" t="inlineStr"/>
@@ -21056,13 +21027,13 @@
           <t>DTD</t>
         </is>
       </c>
-      <c r="J48" s="27" t="n">
+      <c r="J48" s="25" t="n">
         <v>46154.36458333334</v>
       </c>
-      <c r="M48" s="27" t="n">
+      <c r="M48" s="25" t="n">
         <v>46157.43888888889</v>
       </c>
-      <c r="N48" s="27" t="n">
+      <c r="N48" s="25" t="n">
         <v>46021</v>
       </c>
       <c r="Q48" t="inlineStr"/>
@@ -21115,13 +21086,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J49" s="27" t="n">
+      <c r="J49" s="25" t="n">
         <v>46154.37291666667</v>
       </c>
-      <c r="M49" s="27" t="n">
+      <c r="M49" s="25" t="n">
         <v>46205.70069444444</v>
       </c>
-      <c r="N49" s="27" t="n">
+      <c r="N49" s="25" t="n">
         <v>46049</v>
       </c>
       <c r="Q49" t="inlineStr"/>
@@ -21174,16 +21145,16 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="J50" s="27" t="n">
+      <c r="J50" s="25" t="n">
         <v>46154.37152777778</v>
       </c>
-      <c r="M50" s="27" t="n">
+      <c r="M50" s="25" t="n">
         <v>46206.36527777778</v>
       </c>
-      <c r="N50" s="27" t="n">
+      <c r="N50" s="25" t="n">
         <v>46022</v>
       </c>
-      <c r="P50" s="27" t="n">
+      <c r="P50" s="25" t="n">
         <v>46206</v>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -21244,13 +21215,13 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="J51" s="27" t="n">
+      <c r="J51" s="25" t="n">
         <v>46154.36944444444</v>
       </c>
-      <c r="N51" s="27" t="n">
+      <c r="N51" s="25" t="n">
         <v>46017</v>
       </c>
-      <c r="P51" s="27" t="n">
+      <c r="P51" s="25" t="n">
         <v>46206</v>
       </c>
       <c r="Q51" t="inlineStr"/>
@@ -21311,13 +21282,13 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J52" s="27" t="n">
+      <c r="J52" s="25" t="n">
         <v>46154.35625</v>
       </c>
-      <c r="N52" s="27" t="n">
+      <c r="N52" s="25" t="n">
         <v>45934</v>
       </c>
-      <c r="P52" s="27" t="n">
+      <c r="P52" s="25" t="n">
         <v>46206</v>
       </c>
       <c r="Q52" t="inlineStr"/>
@@ -21381,13 +21352,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J53" s="27" t="n">
+      <c r="J53" s="25" t="n">
         <v>46154.35486111111</v>
       </c>
-      <c r="N53" s="27" t="n">
+      <c r="N53" s="25" t="n">
         <v>45973</v>
       </c>
-      <c r="P53" s="27" t="n">
+      <c r="P53" s="25" t="n">
         <v>46206</v>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -21448,13 +21419,13 @@
           <t>DTD</t>
         </is>
       </c>
-      <c r="J54" s="27" t="n">
+      <c r="J54" s="25" t="n">
         <v>46154.36805555555</v>
       </c>
-      <c r="N54" s="27" t="n">
+      <c r="N54" s="25" t="n">
         <v>45938</v>
       </c>
-      <c r="P54" s="27" t="n">
+      <c r="P54" s="25" t="n">
         <v>46206</v>
       </c>
       <c r="Q54" t="inlineStr"/>
@@ -21517,13 +21488,13 @@
           <t>DTD</t>
         </is>
       </c>
-      <c r="J55" s="27" t="n">
+      <c r="J55" s="25" t="n">
         <v>46154.37222222222</v>
       </c>
-      <c r="N55" s="27" t="n">
+      <c r="N55" s="25" t="n">
         <v>46049</v>
       </c>
-      <c r="P55" s="27" t="n">
+      <c r="P55" s="25" t="n">
         <v>46206</v>
       </c>
       <c r="Q55" t="inlineStr"/>
@@ -21579,10 +21550,10 @@
       </c>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="27" t="n">
+      <c r="J56" s="25" t="n">
         <v>46154.38055555556</v>
       </c>
-      <c r="P56" s="27" t="n">
+      <c r="P56" s="25" t="n">
         <v>46206</v>
       </c>
       <c r="Q56" t="inlineStr"/>
@@ -21644,10 +21615,10 @@
           <t>FN</t>
         </is>
       </c>
-      <c r="J57" s="27" t="n">
+      <c r="J57" s="25" t="n">
         <v>46154.37013888889</v>
       </c>
-      <c r="N57" s="27" t="n">
+      <c r="N57" s="25" t="n">
         <v>46052</v>
       </c>
       <c r="Q57" t="inlineStr"/>
@@ -21700,16 +21671,16 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J58" s="27" t="n">
+      <c r="J58" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="L58" s="27" t="n">
+      <c r="L58" s="25" t="n">
         <v>46168.99930555555</v>
       </c>
-      <c r="M58" s="27" t="n">
+      <c r="M58" s="25" t="n">
         <v>46202.59027777778</v>
       </c>
-      <c r="N58" s="27" t="n">
+      <c r="N58" s="25" t="n">
         <v>46049</v>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -21758,13 +21729,13 @@
           <t>ACC</t>
         </is>
       </c>
-      <c r="J59" s="27" t="n">
+      <c r="J59" s="25" t="n">
         <v>46125.71180555555</v>
       </c>
-      <c r="M59" s="27" t="n">
+      <c r="M59" s="25" t="n">
         <v>46202.58958333333</v>
       </c>
-      <c r="N59" s="27" t="n">
+      <c r="N59" s="25" t="n">
         <v>46107</v>
       </c>
       <c r="Q59" t="inlineStr"/>
@@ -21813,13 +21784,13 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="J60" s="27" t="n">
+      <c r="J60" s="25" t="n">
         <v>46125.71805555555</v>
       </c>
-      <c r="M60" s="27" t="n">
+      <c r="M60" s="25" t="n">
         <v>46202.58958333333</v>
       </c>
-      <c r="N60" s="27" t="n">
+      <c r="N60" s="25" t="n">
         <v>46125</v>
       </c>
       <c r="Q60" t="inlineStr"/>
@@ -21872,16 +21843,16 @@
           <t>RS</t>
         </is>
       </c>
-      <c r="J61" s="27" t="n">
+      <c r="J61" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="L61" s="27" t="n">
+      <c r="L61" s="25" t="n">
         <v>46164.99930555555</v>
       </c>
-      <c r="M61" s="27" t="n">
+      <c r="M61" s="25" t="n">
         <v>46178.40555555555</v>
       </c>
-      <c r="N61" s="27" t="n">
+      <c r="N61" s="25" t="n">
         <v>46076</v>
       </c>
       <c r="Q61" t="inlineStr"/>
@@ -21930,13 +21901,13 @@
           <t>INB</t>
         </is>
       </c>
-      <c r="J62" s="27" t="n">
+      <c r="J62" s="25" t="n">
         <v>46121.70833333334</v>
       </c>
-      <c r="M62" s="27" t="n">
+      <c r="M62" s="25" t="n">
         <v>46169.56180555555</v>
       </c>
-      <c r="N62" s="27" t="n">
+      <c r="N62" s="25" t="n">
         <v>46098</v>
       </c>
       <c r="Q62" t="inlineStr"/>
@@ -21981,13 +21952,13 @@
           <t>RS</t>
         </is>
       </c>
-      <c r="J63" s="27" t="n">
+      <c r="J63" s="25" t="n">
         <v>46136.39375</v>
       </c>
-      <c r="M63" s="27" t="n">
+      <c r="M63" s="25" t="n">
         <v>46146.35138888889</v>
       </c>
-      <c r="N63" s="27" t="n">
+      <c r="N63" s="25" t="n">
         <v>46099</v>
       </c>
       <c r="Q63" t="inlineStr"/>
@@ -22040,13 +22011,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J64" s="27" t="n">
+      <c r="J64" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="M64" s="27" t="n">
+      <c r="M64" s="25" t="n">
         <v>46146.34375</v>
       </c>
-      <c r="N64" s="27" t="n">
+      <c r="N64" s="25" t="n">
         <v>46022</v>
       </c>
       <c r="Q64" t="inlineStr"/>
@@ -22095,13 +22066,13 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="J65" s="27" t="n">
+      <c r="J65" s="25" t="n">
         <v>46121.70625</v>
       </c>
-      <c r="M65" s="27" t="n">
+      <c r="M65" s="25" t="n">
         <v>46132.34166666667</v>
       </c>
-      <c r="N65" s="27" t="n">
+      <c r="N65" s="25" t="n">
         <v>46118</v>
       </c>
       <c r="Q65" t="inlineStr"/>
@@ -22154,10 +22125,10 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J66" s="27" t="n">
+      <c r="J66" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="M66" s="27" t="n">
+      <c r="M66" s="25" t="n">
         <v>46132.34097222222</v>
       </c>
       <c r="Q66" t="inlineStr"/>
@@ -22210,13 +22181,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J67" s="27" t="n">
+      <c r="J67" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="M67" s="27" t="n">
+      <c r="M67" s="25" t="n">
         <v>46125.70972222222</v>
       </c>
-      <c r="N67" s="27" t="n">
+      <c r="N67" s="25" t="n">
         <v>46064</v>
       </c>
       <c r="Q67" t="inlineStr"/>
@@ -22269,19 +22240,19 @@
           <t>RMD</t>
         </is>
       </c>
-      <c r="J68" s="27" t="n">
+      <c r="J68" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="K68" s="27" t="n">
+      <c r="K68" s="25" t="n">
         <v>46083</v>
       </c>
-      <c r="L68" s="27" t="n">
+      <c r="L68" s="25" t="n">
         <v>46111.99930555555</v>
       </c>
-      <c r="M68" s="27" t="n">
+      <c r="M68" s="25" t="n">
         <v>46111.625</v>
       </c>
-      <c r="N68" s="27" t="n">
+      <c r="N68" s="25" t="n">
         <v>45952</v>
       </c>
       <c r="Q68" t="inlineStr"/>
@@ -22334,22 +22305,22 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J69" s="27" t="n">
+      <c r="J69" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="K69" s="27" t="n">
+      <c r="K69" s="25" t="n">
         <v>46092</v>
       </c>
-      <c r="L69" s="27" t="n">
+      <c r="L69" s="25" t="n">
         <v>46111.99930555555</v>
       </c>
-      <c r="M69" s="27" t="n">
+      <c r="M69" s="25" t="n">
         <v>46111.625</v>
       </c>
-      <c r="N69" s="27" t="n">
+      <c r="N69" s="25" t="n">
         <v>46021</v>
       </c>
-      <c r="O69" s="27" t="n">
+      <c r="O69" s="25" t="n">
         <v>46080</v>
       </c>
       <c r="Q69" t="inlineStr"/>
@@ -22402,22 +22373,22 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J70" s="27" t="n">
+      <c r="J70" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="K70" s="27" t="n">
+      <c r="K70" s="25" t="n">
         <v>46083</v>
       </c>
-      <c r="L70" s="27" t="n">
+      <c r="L70" s="25" t="n">
         <v>46111.99930555555</v>
       </c>
-      <c r="M70" s="27" t="n">
+      <c r="M70" s="25" t="n">
         <v>46111.62430555555</v>
       </c>
-      <c r="N70" s="27" t="n">
+      <c r="N70" s="25" t="n">
         <v>45986</v>
       </c>
-      <c r="O70" s="27" t="n">
+      <c r="O70" s="25" t="n">
         <v>46056</v>
       </c>
       <c r="Q70" t="inlineStr"/>
@@ -22470,22 +22441,22 @@
           <t>IC</t>
         </is>
       </c>
-      <c r="J71" s="27" t="n">
+      <c r="J71" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="K71" s="27" t="n">
+      <c r="K71" s="25" t="n">
         <v>46084</v>
       </c>
-      <c r="L71" s="27" t="n">
+      <c r="L71" s="25" t="n">
         <v>46097.99930555555</v>
       </c>
-      <c r="M71" s="27" t="n">
+      <c r="M71" s="25" t="n">
         <v>46097.46597222222</v>
       </c>
-      <c r="N71" s="27" t="n">
+      <c r="N71" s="25" t="n">
         <v>46049</v>
       </c>
-      <c r="O71" s="27" t="n">
+      <c r="O71" s="25" t="n">
         <v>46083</v>
       </c>
       <c r="Q71" t="inlineStr"/>
@@ -22538,19 +22509,19 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J72" s="27" t="n">
+      <c r="J72" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="K72" s="27" t="n">
+      <c r="K72" s="25" t="n">
         <v>46079</v>
       </c>
-      <c r="L72" s="27" t="n">
+      <c r="L72" s="25" t="n">
         <v>46097.99930555555</v>
       </c>
-      <c r="M72" s="27" t="n">
+      <c r="M72" s="25" t="n">
         <v>46097.46527777778</v>
       </c>
-      <c r="N72" s="27" t="n">
+      <c r="N72" s="25" t="n">
         <v>46010</v>
       </c>
       <c r="Q72" t="inlineStr"/>
@@ -22603,13 +22574,13 @@
           <t>LG</t>
         </is>
       </c>
-      <c r="J73" s="27" t="n">
+      <c r="J73" s="25" t="n">
         <v>46084.69375</v>
       </c>
-      <c r="M73" s="27" t="n">
+      <c r="M73" s="25" t="n">
         <v>46087.37430555555</v>
       </c>
-      <c r="N73" s="27" t="n">
+      <c r="N73" s="25" t="n">
         <v>46051</v>
       </c>
       <c r="Q73" t="inlineStr"/>
@@ -22662,16 +22633,16 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="J74" s="27" t="n">
+      <c r="J74" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="M74" s="27" t="n">
+      <c r="M74" s="25" t="n">
         <v>46084.69513888889</v>
       </c>
-      <c r="N74" s="27" t="n">
+      <c r="N74" s="25" t="n">
         <v>45982</v>
       </c>
-      <c r="O74" s="27" t="n">
+      <c r="O74" s="25" t="n">
         <v>46064</v>
       </c>
       <c r="Q74" t="inlineStr"/>
@@ -22724,16 +22695,16 @@
           <t>INB</t>
         </is>
       </c>
-      <c r="J75" s="27" t="n">
+      <c r="J75" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="M75" s="27" t="n">
+      <c r="M75" s="25" t="n">
         <v>46084.69513888889</v>
       </c>
-      <c r="N75" s="27" t="n">
+      <c r="N75" s="25" t="n">
         <v>45972</v>
       </c>
-      <c r="O75" s="27" t="n">
+      <c r="O75" s="25" t="n">
         <v>46001</v>
       </c>
       <c r="Q75" t="inlineStr"/>
@@ -22778,13 +22749,13 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="J76" s="27" t="n">
+      <c r="J76" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="M76" s="27" t="n">
+      <c r="M76" s="25" t="n">
         <v>46084.69513888889</v>
       </c>
-      <c r="N76" s="27" t="n">
+      <c r="N76" s="25" t="n">
         <v>46056</v>
       </c>
       <c r="Q76" t="inlineStr"/>
@@ -22837,13 +22808,13 @@
           <t>MKT</t>
         </is>
       </c>
-      <c r="J77" s="27" t="n">
+      <c r="J77" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="M77" s="27" t="n">
+      <c r="M77" s="25" t="n">
         <v>46084.69513888889</v>
       </c>
-      <c r="N77" s="27" t="n">
+      <c r="N77" s="25" t="n">
         <v>45980</v>
       </c>
       <c r="Q77" t="inlineStr"/>
@@ -22896,13 +22867,13 @@
           <t>INB</t>
         </is>
       </c>
-      <c r="J78" s="27" t="n">
+      <c r="J78" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="M78" s="27" t="n">
+      <c r="M78" s="25" t="n">
         <v>46084.69513888889</v>
       </c>
-      <c r="N78" s="27" t="n">
+      <c r="N78" s="25" t="n">
         <v>45942</v>
       </c>
       <c r="Q78" t="inlineStr"/>
@@ -22955,10 +22926,10 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="J79" s="27" t="n">
+      <c r="J79" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="M79" s="27" t="n">
+      <c r="M79" s="25" t="n">
         <v>46084.69513888889</v>
       </c>
       <c r="Q79" t="inlineStr"/>
@@ -23011,13 +22982,13 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="J80" s="27" t="n">
+      <c r="J80" s="25" t="n">
         <v>46084.69444444445</v>
       </c>
-      <c r="M80" s="27" t="n">
+      <c r="M80" s="25" t="n">
         <v>46084.69513888889</v>
       </c>
-      <c r="N80" s="27" t="n">
+      <c r="N80" s="25" t="n">
         <v>45985</v>
       </c>
       <c r="Q80" t="inlineStr"/>
@@ -23070,16 +23041,16 @@
           <t>CCC</t>
         </is>
       </c>
-      <c r="J81" s="27" t="n">
+      <c r="J81" s="25" t="n">
         <v>46084.65763888889</v>
       </c>
-      <c r="M81" s="27" t="n">
+      <c r="M81" s="25" t="n">
         <v>46098.45277777778</v>
       </c>
-      <c r="N81" s="27" t="n">
+      <c r="N81" s="25" t="n">
         <v>46010</v>
       </c>
-      <c r="O81" s="27" t="n">
+      <c r="O81" s="25" t="n">
         <v>46042</v>
       </c>
       <c r="Q81" t="inlineStr"/>
@@ -23132,22 +23103,22 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="J82" s="27" t="n">
+      <c r="J82" s="25" t="n">
         <v>46084.65763888889</v>
       </c>
-      <c r="K82" s="27" t="n">
+      <c r="K82" s="25" t="n">
         <v>46083</v>
       </c>
-      <c r="L82" s="27" t="n">
+      <c r="L82" s="25" t="n">
         <v>46090.99930555555</v>
       </c>
-      <c r="M82" s="27" t="n">
+      <c r="M82" s="25" t="n">
         <v>46091.36597222222</v>
       </c>
-      <c r="N82" s="27" t="n">
+      <c r="N82" s="25" t="n">
         <v>45986</v>
       </c>
-      <c r="O82" s="27" t="n">
+      <c r="O82" s="25" t="n">
         <v>46044</v>
       </c>
       <c r="Q82" t="inlineStr"/>
@@ -23200,16 +23171,16 @@
           <t>MSD</t>
         </is>
       </c>
-      <c r="J83" s="27" t="n">
+      <c r="J83" s="25" t="n">
         <v>46084.65694444445</v>
       </c>
-      <c r="M83" s="27" t="n">
+      <c r="M83" s="25" t="n">
         <v>46085.28888888889</v>
       </c>
-      <c r="N83" s="27" t="n">
+      <c r="N83" s="25" t="n">
         <v>45911</v>
       </c>
-      <c r="O83" s="27" t="n">
+      <c r="O83" s="25" t="n">
         <v>45985</v>
       </c>
       <c r="Q83" t="inlineStr"/>
@@ -23258,16 +23229,16 @@
           <t>BMD</t>
         </is>
       </c>
-      <c r="J84" s="27" t="n">
+      <c r="J84" s="25" t="n">
         <v>46085.68402777778</v>
       </c>
-      <c r="L84" s="27" t="n">
+      <c r="L84" s="25" t="n">
         <v>46066.99930555555</v>
       </c>
-      <c r="M84" s="27" t="n">
+      <c r="M84" s="25" t="n">
         <v>46085.68680555555</v>
       </c>
-      <c r="N84" s="27" t="n">
+      <c r="N84" s="25" t="n">
         <v>45714</v>
       </c>
       <c r="Q84" t="inlineStr"/>
@@ -23289,12 +23260,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>lead_email</t>
         </is>
@@ -23351,17 +23322,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>stage_order</t>
         </is>
       </c>
-      <c r="C1" s="26" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>status_group</t>
         </is>
@@ -23592,12 +23563,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>task_id</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>division</t>
         </is>
@@ -25094,12 +25065,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>task_id</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>platform</t>
         </is>
@@ -26176,12 +26147,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>task_id</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>devunit</t>
         </is>

</xml_diff>